<commit_message>
Add roadmap sheet (18-month risk trajectory, budget) to the workbook, and a management-restitution deck
</commit_message>
<xml_diff>
--- a/reports/SMSI-biotech-classeur.xlsx
+++ b/reports/SMSI-biotech-classeur.xlsx
@@ -1,22 +1,23 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="Lisez-moi" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet name="Socle" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet name="Événements redoutés" sheetId="3" state="visible" r:id="rId3"/>
-    <sheet name="Couples SR-OV" sheetId="4" state="visible" r:id="rId4"/>
-    <sheet name="Parties prenantes" sheetId="5" state="visible" r:id="rId5"/>
-    <sheet name="Risques" sheetId="6" state="visible" r:id="rId6"/>
-    <sheet name="Modes opératoires" sheetId="7" state="visible" r:id="rId7"/>
-    <sheet name="Plan de traitement" sheetId="8" state="visible" r:id="rId8"/>
-    <sheet name="Déclaration d'applicabilité" sheetId="9" state="visible" r:id="rId9"/>
-    <sheet name="Indicateurs" sheetId="10" state="visible" r:id="rId10"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Lisez-moi" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Socle" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Événements redoutés" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Couples SR-OV" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Parties prenantes" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Risques" sheetId="6" state="visible" r:id="rId6"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Modes opératoires" sheetId="7" state="visible" r:id="rId7"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Plan de traitement" sheetId="8" state="visible" r:id="rId8"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Déclaration d'applicabilité" sheetId="9" state="visible" r:id="rId9"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Indicateurs" sheetId="10" state="visible" r:id="rId10"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Trajectoire" sheetId="11" state="visible" r:id="rId11"/>
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Socle'!$A$1:$H$43</definedName>
@@ -28,6 +29,7 @@
     <definedName name="_xlnm._FilterDatabase" localSheetId="7" hidden="1">'Plan de traitement'!$A$1:$O$27</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="8" hidden="1">'Déclaration d''applicabilité'!$A$1:$J$94</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="9" hidden="1">'Indicateurs'!$A$1:$H$14</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="10" hidden="1">'Trajectoire'!$A$1:$L$8</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -36,7 +38,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="3">
+  <fonts count="5">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -50,6 +52,13 @@
     </font>
     <font>
       <b val="1"/>
+    </font>
+    <font>
+      <b val="1"/>
+      <sz val="12"/>
+    </font>
+    <font>
+      <i val="1"/>
     </font>
   </fonts>
   <fills count="3">
@@ -77,7 +86,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="4">
+  <cellXfs count="8">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
@@ -86,6 +95,10 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="2" fillId="2" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -1133,6 +1146,612 @@
 </worksheet>
 </file>
 
+<file path=xl/worksheets/sheet11.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:L17"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="26" customWidth="1" min="1" max="1"/>
+    <col width="12" customWidth="1" min="2" max="2"/>
+    <col width="13" customWidth="1" min="3" max="3"/>
+    <col width="13" customWidth="1" min="4" max="4"/>
+    <col width="13" customWidth="1" min="5" max="5"/>
+    <col width="13" customWidth="1" min="6" max="6"/>
+    <col width="13" customWidth="1" min="7" max="7"/>
+    <col width="13" customWidth="1" min="8" max="8"/>
+    <col width="13" customWidth="1" min="9" max="9"/>
+    <col width="13" customWidth="1" min="10" max="10"/>
+    <col width="13" customWidth="1" min="11" max="11"/>
+    <col width="13" customWidth="1" min="12" max="12"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="2" t="inlineStr">
+        <is>
+          <t>Réf.</t>
+        </is>
+      </c>
+      <c r="B1" s="2" t="inlineStr">
+        <is>
+          <t>Score initial</t>
+        </is>
+      </c>
+      <c r="C1" s="2" t="inlineStr">
+        <is>
+          <t>T0 (aujourd'hui)</t>
+        </is>
+      </c>
+      <c r="D1" s="2" t="inlineStr">
+        <is>
+          <t>Niveau</t>
+        </is>
+      </c>
+      <c r="E1" s="2" t="inlineStr">
+        <is>
+          <t>T0+6 mois</t>
+        </is>
+      </c>
+      <c r="F1" s="2" t="inlineStr">
+        <is>
+          <t>Niveau</t>
+        </is>
+      </c>
+      <c r="G1" s="2" t="inlineStr">
+        <is>
+          <t>T0+12 mois</t>
+        </is>
+      </c>
+      <c r="H1" s="2" t="inlineStr">
+        <is>
+          <t>Niveau</t>
+        </is>
+      </c>
+      <c r="I1" s="2" t="inlineStr">
+        <is>
+          <t>T0+18 mois</t>
+        </is>
+      </c>
+      <c r="J1" s="2" t="inlineStr">
+        <is>
+          <t>Niveau</t>
+        </is>
+      </c>
+      <c r="K1" s="2" t="inlineStr">
+        <is>
+          <t>Score cible</t>
+        </is>
+      </c>
+      <c r="L1" s="2" t="inlineStr">
+        <is>
+          <t>Niveau cible</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>R1</t>
+        </is>
+      </c>
+      <c r="B2" t="n">
+        <v>9</v>
+      </c>
+      <c r="C2" t="n">
+        <v>8.699999999999999</v>
+      </c>
+      <c r="D2">
+        <f>IF(C2&gt;=8,"Élevé",IF(C2&gt;=4,"Moyen","Faible"))</f>
+        <v/>
+      </c>
+      <c r="E2" t="n">
+        <v>7.2</v>
+      </c>
+      <c r="F2">
+        <f>IF(E2&gt;=8,"Élevé",IF(E2&gt;=4,"Moyen","Faible"))</f>
+        <v/>
+      </c>
+      <c r="G2" t="n">
+        <v>6</v>
+      </c>
+      <c r="H2">
+        <f>IF(G2&gt;=8,"Élevé",IF(G2&gt;=4,"Moyen","Faible"))</f>
+        <v/>
+      </c>
+      <c r="I2" t="n">
+        <v>6</v>
+      </c>
+      <c r="J2">
+        <f>IF(I2&gt;=8,"Élevé",IF(I2&gt;=4,"Moyen","Faible"))</f>
+        <v/>
+      </c>
+      <c r="K2" t="n">
+        <v>6</v>
+      </c>
+      <c r="L2">
+        <f>IF(K2&gt;=8,"Élevé",IF(K2&gt;=4,"Moyen","Faible"))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>R2</t>
+        </is>
+      </c>
+      <c r="B3" t="n">
+        <v>6</v>
+      </c>
+      <c r="C3" t="n">
+        <v>5.5</v>
+      </c>
+      <c r="D3">
+        <f>IF(C3&gt;=8,"Élevé",IF(C3&gt;=4,"Moyen","Faible"))</f>
+        <v/>
+      </c>
+      <c r="E3" t="n">
+        <v>4</v>
+      </c>
+      <c r="F3">
+        <f>IF(E3&gt;=8,"Élevé",IF(E3&gt;=4,"Moyen","Faible"))</f>
+        <v/>
+      </c>
+      <c r="G3" t="n">
+        <v>3.5</v>
+      </c>
+      <c r="H3">
+        <f>IF(G3&gt;=8,"Élevé",IF(G3&gt;=4,"Moyen","Faible"))</f>
+        <v/>
+      </c>
+      <c r="I3" t="n">
+        <v>3</v>
+      </c>
+      <c r="J3">
+        <f>IF(I3&gt;=8,"Élevé",IF(I3&gt;=4,"Moyen","Faible"))</f>
+        <v/>
+      </c>
+      <c r="K3" t="n">
+        <v>3</v>
+      </c>
+      <c r="L3">
+        <f>IF(K3&gt;=8,"Élevé",IF(K3&gt;=4,"Moyen","Faible"))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>R3</t>
+        </is>
+      </c>
+      <c r="B4" t="n">
+        <v>12</v>
+      </c>
+      <c r="C4" t="n">
+        <v>12</v>
+      </c>
+      <c r="D4">
+        <f>IF(C4&gt;=8,"Élevé",IF(C4&gt;=4,"Moyen","Faible"))</f>
+        <v/>
+      </c>
+      <c r="E4" t="n">
+        <v>10</v>
+      </c>
+      <c r="F4">
+        <f>IF(E4&gt;=8,"Élevé",IF(E4&gt;=4,"Moyen","Faible"))</f>
+        <v/>
+      </c>
+      <c r="G4" t="n">
+        <v>9.300000000000001</v>
+      </c>
+      <c r="H4">
+        <f>IF(G4&gt;=8,"Élevé",IF(G4&gt;=4,"Moyen","Faible"))</f>
+        <v/>
+      </c>
+      <c r="I4" t="n">
+        <v>9</v>
+      </c>
+      <c r="J4">
+        <f>IF(I4&gt;=8,"Élevé",IF(I4&gt;=4,"Moyen","Faible"))</f>
+        <v/>
+      </c>
+      <c r="K4" t="n">
+        <v>9</v>
+      </c>
+      <c r="L4">
+        <f>IF(K4&gt;=8,"Élevé",IF(K4&gt;=4,"Moyen","Faible"))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>R4</t>
+        </is>
+      </c>
+      <c r="B5" t="n">
+        <v>8</v>
+      </c>
+      <c r="C5" t="n">
+        <v>8</v>
+      </c>
+      <c r="D5">
+        <f>IF(C5&gt;=8,"Élevé",IF(C5&gt;=4,"Moyen","Faible"))</f>
+        <v/>
+      </c>
+      <c r="E5" t="n">
+        <v>5.6</v>
+      </c>
+      <c r="F5">
+        <f>IF(E5&gt;=8,"Élevé",IF(E5&gt;=4,"Moyen","Faible"))</f>
+        <v/>
+      </c>
+      <c r="G5" t="n">
+        <v>4.4</v>
+      </c>
+      <c r="H5">
+        <f>IF(G5&gt;=8,"Élevé",IF(G5&gt;=4,"Moyen","Faible"))</f>
+        <v/>
+      </c>
+      <c r="I5" t="n">
+        <v>4</v>
+      </c>
+      <c r="J5">
+        <f>IF(I5&gt;=8,"Élevé",IF(I5&gt;=4,"Moyen","Faible"))</f>
+        <v/>
+      </c>
+      <c r="K5" t="n">
+        <v>4</v>
+      </c>
+      <c r="L5">
+        <f>IF(K5&gt;=8,"Élevé",IF(K5&gt;=4,"Moyen","Faible"))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>R5</t>
+        </is>
+      </c>
+      <c r="B6" t="n">
+        <v>4</v>
+      </c>
+      <c r="C6" t="n">
+        <v>4</v>
+      </c>
+      <c r="D6">
+        <f>IF(C6&gt;=8,"Élevé",IF(C6&gt;=4,"Moyen","Faible"))</f>
+        <v/>
+      </c>
+      <c r="E6" t="n">
+        <v>3.4</v>
+      </c>
+      <c r="F6">
+        <f>IF(E6&gt;=8,"Élevé",IF(E6&gt;=4,"Moyen","Faible"))</f>
+        <v/>
+      </c>
+      <c r="G6" t="n">
+        <v>3</v>
+      </c>
+      <c r="H6">
+        <f>IF(G6&gt;=8,"Élevé",IF(G6&gt;=4,"Moyen","Faible"))</f>
+        <v/>
+      </c>
+      <c r="I6" t="n">
+        <v>3</v>
+      </c>
+      <c r="J6">
+        <f>IF(I6&gt;=8,"Élevé",IF(I6&gt;=4,"Moyen","Faible"))</f>
+        <v/>
+      </c>
+      <c r="K6" t="n">
+        <v>3</v>
+      </c>
+      <c r="L6">
+        <f>IF(K6&gt;=8,"Élevé",IF(K6&gt;=4,"Moyen","Faible"))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>R6</t>
+        </is>
+      </c>
+      <c r="B7" t="n">
+        <v>16</v>
+      </c>
+      <c r="C7" t="n">
+        <v>16</v>
+      </c>
+      <c r="D7">
+        <f>IF(C7&gt;=8,"Élevé",IF(C7&gt;=4,"Moyen","Faible"))</f>
+        <v/>
+      </c>
+      <c r="E7" t="n">
+        <v>9.9</v>
+      </c>
+      <c r="F7">
+        <f>IF(E7&gt;=8,"Élevé",IF(E7&gt;=4,"Moyen","Faible"))</f>
+        <v/>
+      </c>
+      <c r="G7" t="n">
+        <v>6.6</v>
+      </c>
+      <c r="H7">
+        <f>IF(G7&gt;=8,"Élevé",IF(G7&gt;=4,"Moyen","Faible"))</f>
+        <v/>
+      </c>
+      <c r="I7" t="n">
+        <v>6</v>
+      </c>
+      <c r="J7">
+        <f>IF(I7&gt;=8,"Élevé",IF(I7&gt;=4,"Moyen","Faible"))</f>
+        <v/>
+      </c>
+      <c r="K7" t="n">
+        <v>6</v>
+      </c>
+      <c r="L7">
+        <f>IF(K7&gt;=8,"Élevé",IF(K7&gt;=4,"Moyen","Faible"))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>R7</t>
+        </is>
+      </c>
+      <c r="B8" t="n">
+        <v>12</v>
+      </c>
+      <c r="C8" t="n">
+        <v>12</v>
+      </c>
+      <c r="D8">
+        <f>IF(C8&gt;=8,"Élevé",IF(C8&gt;=4,"Moyen","Faible"))</f>
+        <v/>
+      </c>
+      <c r="E8" t="n">
+        <v>8.4</v>
+      </c>
+      <c r="F8">
+        <f>IF(E8&gt;=8,"Élevé",IF(E8&gt;=4,"Moyen","Faible"))</f>
+        <v/>
+      </c>
+      <c r="G8" t="n">
+        <v>6</v>
+      </c>
+      <c r="H8">
+        <f>IF(G8&gt;=8,"Élevé",IF(G8&gt;=4,"Moyen","Faible"))</f>
+        <v/>
+      </c>
+      <c r="I8" t="n">
+        <v>6</v>
+      </c>
+      <c r="J8">
+        <f>IF(I8&gt;=8,"Élevé",IF(I8&gt;=4,"Moyen","Faible"))</f>
+        <v/>
+      </c>
+      <c r="K8" t="n">
+        <v>6</v>
+      </c>
+      <c r="L8">
+        <f>IF(K8&gt;=8,"Élevé",IF(K8&gt;=4,"Moyen","Faible"))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="4" t="inlineStr">
+        <is>
+          <t>Moyenne</t>
+        </is>
+      </c>
+      <c r="B9" s="4">
+        <f>AVERAGE(B2:B8)</f>
+        <v/>
+      </c>
+      <c r="C9" s="4">
+        <f>AVERAGE(C2:C8)</f>
+        <v/>
+      </c>
+      <c r="D9" s="4" t="inlineStr"/>
+      <c r="E9" s="4">
+        <f>AVERAGE(E2:E8)</f>
+        <v/>
+      </c>
+      <c r="F9" s="4" t="inlineStr"/>
+      <c r="G9" s="4">
+        <f>AVERAGE(G2:G8)</f>
+        <v/>
+      </c>
+      <c r="H9" s="4" t="inlineStr"/>
+      <c r="I9" s="4">
+        <f>AVERAGE(I2:I8)</f>
+        <v/>
+      </c>
+      <c r="J9" s="4" t="inlineStr"/>
+      <c r="K9" s="4">
+        <f>AVERAGE(K2:K8)</f>
+        <v/>
+      </c>
+      <c r="L9" s="4" t="inlineStr"/>
+    </row>
+    <row r="10">
+      <c r="A10" s="4" t="inlineStr">
+        <is>
+          <t>Risques au niveau Élevé</t>
+        </is>
+      </c>
+      <c r="B10" s="4">
+        <f>COUNTIF(D2:D8,"Élevé")</f>
+        <v/>
+      </c>
+      <c r="C10" s="4" t="inlineStr"/>
+      <c r="D10" s="4" t="inlineStr"/>
+      <c r="E10" s="4">
+        <f>COUNTIF(F2:F8,"Élevé")</f>
+        <v/>
+      </c>
+      <c r="F10" s="4" t="inlineStr"/>
+      <c r="G10" s="4">
+        <f>COUNTIF(H2:H8,"Élevé")</f>
+        <v/>
+      </c>
+      <c r="H10" s="4" t="inlineStr"/>
+      <c r="I10" s="4">
+        <f>COUNTIF(J2:J8,"Élevé")</f>
+        <v/>
+      </c>
+      <c r="J10" s="4" t="inlineStr"/>
+      <c r="K10" s="4">
+        <f>COUNTIF(L2:L8,"Élevé")</f>
+        <v/>
+      </c>
+      <c r="L10" s="4" t="inlineStr"/>
+    </row>
+    <row r="12">
+      <c r="A12" s="5" t="inlineStr">
+        <is>
+          <t>Enveloppe budgétaire estimée (mesures restant à réaliser : 24 sur 26)</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="6" t="inlineStr">
+        <is>
+          <t>Priorité</t>
+        </is>
+      </c>
+      <c r="B13" s="6" t="inlineStr">
+        <is>
+          <t>Mesures</t>
+        </is>
+      </c>
+      <c r="C13" s="6" t="inlineStr">
+        <is>
+          <t>Budget</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>P1</t>
+        </is>
+      </c>
+      <c r="B14" t="n">
+        <v>14</v>
+      </c>
+      <c r="C14" t="inlineStr">
+        <is>
+          <t>230 à 1030 k€</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="inlineStr">
+        <is>
+          <t>P2</t>
+        </is>
+      </c>
+      <c r="B15" t="n">
+        <v>8</v>
+      </c>
+      <c r="C15" t="inlineStr">
+        <is>
+          <t>150 à 660 k€</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="inlineStr">
+        <is>
+          <t>P3</t>
+        </is>
+      </c>
+      <c r="B16" t="n">
+        <v>2</v>
+      </c>
+      <c r="C16" t="inlineStr">
+        <is>
+          <t>0 à 20 k€</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="7" t="inlineStr">
+        <is>
+          <t>Total : entre 380 et 1710 k€, et 305 jours-hommes chiffrés</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <autoFilter ref="A1:L8"/>
+  <conditionalFormatting sqref="D2:D8">
+    <cfRule type="cellIs" priority="1" operator="equal" dxfId="2">
+      <formula>"Élevé"</formula>
+    </cfRule>
+    <cfRule type="cellIs" priority="2" operator="equal" dxfId="1">
+      <formula>"Moyen"</formula>
+    </cfRule>
+    <cfRule type="cellIs" priority="3" operator="equal" dxfId="0">
+      <formula>"Faible"</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="F2:F8">
+    <cfRule type="cellIs" priority="4" operator="equal" dxfId="2">
+      <formula>"Élevé"</formula>
+    </cfRule>
+    <cfRule type="cellIs" priority="5" operator="equal" dxfId="1">
+      <formula>"Moyen"</formula>
+    </cfRule>
+    <cfRule type="cellIs" priority="6" operator="equal" dxfId="0">
+      <formula>"Faible"</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="H2:H8">
+    <cfRule type="cellIs" priority="7" operator="equal" dxfId="2">
+      <formula>"Élevé"</formula>
+    </cfRule>
+    <cfRule type="cellIs" priority="8" operator="equal" dxfId="1">
+      <formula>"Moyen"</formula>
+    </cfRule>
+    <cfRule type="cellIs" priority="9" operator="equal" dxfId="0">
+      <formula>"Faible"</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="J2:J8">
+    <cfRule type="cellIs" priority="10" operator="equal" dxfId="2">
+      <formula>"Élevé"</formula>
+    </cfRule>
+    <cfRule type="cellIs" priority="11" operator="equal" dxfId="1">
+      <formula>"Moyen"</formula>
+    </cfRule>
+    <cfRule type="cellIs" priority="12" operator="equal" dxfId="0">
+      <formula>"Faible"</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="L2:L8">
+    <cfRule type="cellIs" priority="13" operator="equal" dxfId="2">
+      <formula>"Élevé"</formula>
+    </cfRule>
+    <cfRule type="cellIs" priority="14" operator="equal" dxfId="1">
+      <formula>"Moyen"</formula>
+    </cfRule>
+    <cfRule type="cellIs" priority="15" operator="equal" dxfId="0">
+      <formula>"Faible"</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>

</xml_diff>